<commit_message>
excel file edit test
text added next to game title
</commit_message>
<xml_diff>
--- a/Documents/MidtermTeamInfoSheet.xlsx
+++ b/Documents/MidtermTeamInfoSheet.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" autoCompressPictures="0" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ADBDC33-2B68-48E6-8BA0-CE99A091F28B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1FBBCBD-772F-40FB-B89F-9DA371C124E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12165" yWindow="0" windowWidth="16740" windowHeight="15585" tabRatio="629" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5184" yWindow="1884" windowWidth="13980" windowHeight="9960" tabRatio="629" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Team info" sheetId="18" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="53">
   <si>
     <t>Team Name</t>
   </si>
@@ -181,6 +181,9 @@
   </si>
   <si>
     <t>Miguel Flores</t>
+  </si>
+  <si>
+    <t>fas;dlkfj;asldkjf</t>
   </si>
 </sst>
 </file>
@@ -729,25 +732,28 @@
     <tabColor theme="0" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="30.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="30.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="48.85546875" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="37.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="28.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="30.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="30.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="48.88671875" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="18" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="12" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="C1" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>13</v>
       </c>
@@ -755,7 +761,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>14</v>
       </c>
@@ -763,8 +769,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:5" ht="19.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:5" ht="18.600000000000001" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -781,7 +787,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="14.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
         <v>33</v>
       </c>
@@ -798,7 +804,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="13.8" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>29</v>
       </c>
@@ -815,7 +821,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
         <v>50</v>
       </c>
@@ -832,7 +838,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
         <v>49</v>
       </c>
@@ -849,7 +855,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
         <v>51</v>
       </c>
@@ -866,7 +872,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
         <v>46</v>
       </c>
@@ -883,41 +889,41 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
       <c r="E12" s="7"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="15"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
       <c r="E13" s="7"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
     </row>
-    <row r="15" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="17"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
     </row>
-    <row r="16" spans="1:5" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="1:5" ht="19.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" ht="14.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="17" spans="1:5" ht="18.600000000000001" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="19.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" ht="18.600000000000001" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>2</v>
       </c>
@@ -934,7 +940,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" ht="13.8" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>17</v>
       </c>
@@ -951,7 +957,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
         <v>18</v>
       </c>
@@ -966,7 +972,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
         <v>16</v>
       </c>

</xml_diff>